<commit_message>
Excel sheets updated for BM, SM
</commit_message>
<xml_diff>
--- a/data/source_files/3. BM - IE3.xlsx
+++ b/data/source_files/3. BM - IE3.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="207">
   <si>
     <t>Motor Type</t>
   </si>
@@ -769,6 +769,27 @@
   </si>
   <si>
     <t>Thermal withstand curve</t>
+  </si>
+  <si>
+    <t>2.43 / 1.41</t>
+  </si>
+  <si>
+    <t>14 / 8.4</t>
+  </si>
+  <si>
+    <t>19.1 / 11.1</t>
+  </si>
+  <si>
+    <t>26.0 / 15.0</t>
+  </si>
+  <si>
+    <t>37.7 / 21.8</t>
+  </si>
+  <si>
+    <t>72.5 / 41.7</t>
+  </si>
+  <si>
+    <t>137.9 / 79.3</t>
   </si>
 </sst>
 </file>
@@ -2766,7 +2787,7 @@
         <v>40</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>39</v>
+        <v>200</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>41</v>
@@ -2781,16 +2802,16 @@
         <v>44</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>45</v>
+        <v>201</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>47</v>
+        <v>203</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>48</v>
+        <v>204</v>
       </c>
       <c r="Q9" s="8" t="s">
         <v>49</v>
@@ -2799,7 +2820,7 @@
         <v>50</v>
       </c>
       <c r="S9" s="8" t="s">
-        <v>51</v>
+        <v>205</v>
       </c>
       <c r="T9" s="8" t="s">
         <v>52</v>
@@ -2808,7 +2829,7 @@
         <v>53</v>
       </c>
       <c r="V9" s="8" t="s">
-        <v>54</v>
+        <v>206</v>
       </c>
       <c r="W9" s="8" t="s">
         <v>55</v>
@@ -2840,8 +2861,8 @@
       <c r="G10" s="11">
         <v>1415</v>
       </c>
-      <c r="H10" s="10" t="s">
-        <v>39</v>
+      <c r="H10" s="10">
+        <v>1408</v>
       </c>
       <c r="I10" s="8">
         <v>1415</v>
@@ -2856,7 +2877,7 @@
         <v>1440</v>
       </c>
       <c r="M10" s="8">
-        <v>1450</v>
+        <v>1445</v>
       </c>
       <c r="N10" s="8">
         <v>1457</v>
@@ -2915,14 +2936,14 @@
       <c r="G11" s="11">
         <v>2.6</v>
       </c>
-      <c r="H11" s="10" t="s">
-        <v>39</v>
+      <c r="H11" s="10">
+        <v>3.7</v>
       </c>
       <c r="I11" s="8">
-        <v>5.06</v>
+        <v>5.1</v>
       </c>
       <c r="J11" s="8">
-        <v>7.37</v>
+        <v>7.4</v>
       </c>
       <c r="K11" s="8">
         <v>10</v>
@@ -2931,13 +2952,13 @@
         <v>14.5</v>
       </c>
       <c r="M11" s="8">
-        <v>24.2</v>
+        <v>26.4</v>
       </c>
       <c r="N11" s="12">
-        <v>36</v>
+        <v>36.1</v>
       </c>
       <c r="O11" s="8">
-        <v>49.2</v>
+        <v>49.3</v>
       </c>
       <c r="P11" s="8">
         <v>71.9</v>
@@ -3371,10 +3392,10 @@
         <v>33.6</v>
       </c>
       <c r="M17" s="8">
-        <v>7.1</v>
+        <v>66.4</v>
       </c>
       <c r="N17" s="8">
-        <v>66.4</v>
+        <v>86.6</v>
       </c>
       <c r="O17" s="8">
         <v>109.5</v>
@@ -3446,10 +3467,10 @@
         <v>42.1</v>
       </c>
       <c r="M18" s="8">
-        <v>3.7</v>
+        <v>122</v>
       </c>
       <c r="N18" s="8">
-        <v>122</v>
+        <v>122.7</v>
       </c>
       <c r="O18" s="8">
         <v>172.6</v>
@@ -3521,10 +3542,10 @@
         <v>45</v>
       </c>
       <c r="M19" s="8">
-        <v>4.5</v>
+        <v>132.5</v>
       </c>
       <c r="N19" s="8">
-        <v>132.5</v>
+        <v>130</v>
       </c>
       <c r="O19" s="17">
         <v>167.6</v>
@@ -3596,10 +3617,10 @@
         <v>86.7</v>
       </c>
       <c r="M20" s="8">
-        <v>88.8</v>
+        <v>88.6</v>
       </c>
       <c r="N20" s="8">
-        <v>88.6</v>
+        <v>89.6</v>
       </c>
       <c r="O20" s="8">
         <v>90.4</v>
@@ -3669,10 +3690,10 @@
         <v>87</v>
       </c>
       <c r="M21" s="8">
-        <v>88.9</v>
+        <v>88.8</v>
       </c>
       <c r="N21" s="8">
-        <v>88.8</v>
+        <v>91.1</v>
       </c>
       <c r="O21" s="8">
         <v>90.7</v>
@@ -3745,7 +3766,7 @@
         <v>87.6</v>
       </c>
       <c r="N22" s="8">
-        <v>87.6</v>
+        <v>89.3</v>
       </c>
       <c r="O22" s="8">
         <v>90.2</v>
@@ -3817,10 +3838,10 @@
         <v>0.76</v>
       </c>
       <c r="M23" s="28">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="N23" s="28">
-        <v>0.77</v>
+        <v>0.82</v>
       </c>
       <c r="O23" s="28">
         <v>0.82</v>
@@ -3890,10 +3911,10 @@
         <v>0.67</v>
       </c>
       <c r="M24" s="28">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="N24" s="28">
-        <v>0.67</v>
+        <v>0.77</v>
       </c>
       <c r="O24" s="28">
         <v>0.72</v>
@@ -3963,10 +3984,10 @@
         <v>0.54</v>
       </c>
       <c r="M25" s="28">
-        <v>0.54</v>
+        <v>0.52</v>
       </c>
       <c r="N25" s="28">
-        <v>0.52</v>
+        <v>0.65</v>
       </c>
       <c r="O25" s="28">
         <v>0.61</v>
@@ -4337,7 +4358,7 @@
         <v>92</v>
       </c>
       <c r="N30" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O30" s="8" t="s">
         <v>93</v>
@@ -4410,13 +4431,13 @@
         <v>92</v>
       </c>
       <c r="N31" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O31" s="8" t="s">
         <v>93</v>
       </c>
       <c r="P31" s="8" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="Q31" s="8" t="s">
         <v>95</v>
@@ -4781,7 +4802,7 @@
         <v>37</v>
       </c>
       <c r="N36" s="11">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="O36" s="34">
         <v>71</v>
@@ -5154,7 +5175,7 @@
         <v>126</v>
       </c>
       <c r="P41" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q41" s="8" t="s">
         <v>127</v>
@@ -5300,19 +5321,19 @@
         <v>130</v>
       </c>
       <c r="P43" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="Q43" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="R43" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="S43" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="T43" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="U43" s="8" t="s">
         <v>131</v>
@@ -5367,7 +5388,7 @@
         <v>133</v>
       </c>
       <c r="N44" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O44" s="8" t="s">
         <v>134</v>
@@ -5939,7 +5960,7 @@
         <v>168</v>
       </c>
       <c r="H52" s="44" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I52" s="44" t="s">
         <v>168</v>
@@ -6222,55 +6243,55 @@
       <c r="E56" s="10"/>
       <c r="F56" s="10"/>
       <c r="G56" s="11">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="H56" s="34">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="I56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="J56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="K56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="L56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="M56" s="8">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="N56" s="8">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="O56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="P56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="Q56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="R56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="S56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="T56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="U56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="V56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="W56" s="17">
-        <v>415</v>
+        <v>240</v>
       </c>
       <c r="X56" s="9"/>
       <c r="Y56" s="9"/>
@@ -6358,55 +6379,55 @@
       <c r="E58" s="10"/>
       <c r="F58" s="10"/>
       <c r="G58" s="11">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="H58" s="34">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="I58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="J58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="K58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="L58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="M58" s="8">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="N58" s="8">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="O58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="P58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="Q58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="R58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="S58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="T58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="U58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="V58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="W58" s="17">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="X58" s="9"/>
       <c r="Y58" s="9"/>
@@ -6542,7 +6563,7 @@
         <v>1.4</v>
       </c>
       <c r="W60" s="17">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="X60" s="9"/>
       <c r="Y60" s="9"/>
@@ -6578,7 +6599,7 @@
         <v>180</v>
       </c>
       <c r="L61" s="17">
-        <v>255</v>
+        <v>225</v>
       </c>
       <c r="M61" s="8">
         <v>290</v>

</xml_diff>